<commit_message>
Dept-specific curriculum: CSE=Networks/OS, IT=WebTech/DBMS, ADS=Python Analytics/StatML, AIML=AI/DeepLearning
</commit_message>
<xml_diff>
--- a/backend/Courses.xlsx
+++ b/backend/Courses.xlsx
@@ -487,7 +487,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>The Network Core, Circuit switching and packet switching, Delay, Loss and throughput in packet switched networks</t>
+          <t>The Network Core, Circuit Switching and Packet Switching, Delay, Loss and Throughput in Packet Switched Networks</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -510,7 +510,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Protocol Layers and their Service Models, IP stack, OSI Model</t>
+          <t>Protocol Layers and their Service Models, IP Stack, OSI Model</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -533,7 +533,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Introduction to principles of Network Applications, The Web and HTTP types Persistent and Non-persistent</t>
+          <t>Introduction to Network Applications, The Web, HTTP, Persistent and Non-Persistent Connections</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -556,7 +556,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Basic Networking Commands, Socket programming in Java</t>
+          <t>Basic Networking Commands, Socket Programming in Java</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -579,7 +579,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Introduction to the Network, The Internet, The Network Edge, Network Topology, Types of Networks, The Network Core, Circuit switching and packet switching, Delay, Loss and throughput in packet switched networks, Protocol Layers and their Service Models, IP stack, OSI Model</t>
+          <t>Introduction to the Network, The Internet, Network Edge, Network Topology, Network Core, Circuit and Packet Switching, Protocol Layers, OSI Model</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -602,7 +602,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Introduction to the Network, The Internet, The Network Edge, Network Topology, Types of Networks, The Network Core, Circuit switching and packet switching, Delay, Loss and throughput in packet switched networks, Protocol Layers and their Service Models, IP stack, OSI Model, Introduction to principles of Network Applications, The Web and HTTP types Persistent and Non-persistent, FTP, Electronic Mail in the Internet with SMTP, POP3 and IMAP protocol, DNS - Routing, Caching</t>
+          <t>All Units: Network Fundamentals, Packet Switching, OSI/IP Layers, HTTP, DNS, FTP, Email Protocols, SMTP, POP3, IMAP, Transport Layer, TCP, UDP, Congestion Control</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -622,7 +622,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C9"/>
+  <dimension ref="A1:D9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -638,6 +638,11 @@
       </c>
       <c r="C1" t="inlineStr">
         <is>
+          <t>Curriculum</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
           <t>Strategies</t>
         </is>
       </c>
@@ -652,6 +657,11 @@
         <v>10</v>
       </c>
       <c r="C2" t="inlineStr">
+        <is>
+          <t>Introduction to Operating Systems, Process Concepts, Process States, Process Control Block (PCB), Context Switching</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
         <is>
           <t>Step 1: Re-read the topic from your lecture notes and highlight the 3 most important concepts.
 Step 2: Look up 2-3 solved examples from your textbook that are similar to the assignment problem.
@@ -672,6 +682,11 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
+          <t>CPU Scheduling Algorithms: FCFS, SJF, Round Robin, Priority Scheduling, Multilevel Queue Scheduling, Gantt Charts</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
           <t>Step 1: Carefully re-read the problem statement and underline the key requirements.
 Step 2: Identify which algorithm, concept, or formula is being tested in this assignment.
 Step 3: Write pseudo-code or a rough outline before writing your actual solution.
@@ -691,6 +706,11 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
+          <t>Process Synchronization, Critical Section Problem, Mutex Locks, Semaphores, Monitors</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
           <t>Step 1: List all topics covered in class since the course started and create a quick topic checklist.
 Step 2: Make flashcards for key definitions, formulas, and important terms for each topic.
 Step 3: Solve at least 4-5 practice questions per topic from your textbook or past quizzes.
@@ -710,6 +730,11 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
+          <t>Deadlocks: Necessary Conditions, Prevention, Avoidance, Detection and Recovery, Banker's Algorithm</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
           <t>Step 1: Review your Quiz 1 paper and fix every mistake to understand why you went wrong.
 Step 2: Focus on the current topic: write out the key algorithm or concept from memory twice.
 Step 3: Implement the required algorithm or technique in code and run it to verify correctness.
@@ -729,6 +754,11 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
+          <t>Memory Management: Paging, Segmentation, Virtual Memory, Page Replacement Algorithms (FIFO, LRU, Optimal)</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
           <t>Step 1: Draw diagrams or visual representations for each concept covered since Quiz 2.
 Step 2: Trace through at least 2 worked examples step-by-step for each key topic.
 Step 3: Code up at least 2 implementations from scratch without looking at your notes.
@@ -747,6 +777,11 @@
         <v>30</v>
       </c>
       <c r="C7" t="inlineStr">
+        <is>
+          <t>CPU Scheduling Simulation using C/Java, POSIX Thread Programming, Semaphore Exercises</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
         <is>
           <t>Step 1: Go through all lab exercises from the semester and redo the ones you found difficult.
 Step 2: Practice writing code entirely from scratch for the most common lab tasks without copy-paste.
@@ -768,6 +803,11 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
+          <t>OS Introduction, Process Management, CPU Scheduling, Process Synchronization, Deadlock Handling</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
           <t>Step 1: Create a one-page topic summary for every chapter or unit covered so far.
 Step 2: Attempt 2 complete past mid-exam papers under strict timed conditions.
 Step 3: Identify your 3 weakest topics from the mock attempts and spend extra time on them.
@@ -787,6 +827,11 @@
         <v>100</v>
       </c>
       <c r="C9" t="inlineStr">
+        <is>
+          <t>Complete OS: Process Management, CPU Scheduling, Synchronization, Deadlocks, Memory Management, File Systems, I/O Management, Protection and Security</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
         <is>
           <t>Step 1: Build a 2-week revision schedule that covers every topic with more time for weak areas.
 Step 2: Prioritize topics by their exam weight and your current performance from your marks data.
@@ -853,7 +898,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Introduction to the Network, The Internet, The Network Edge, Network Topology, Types of Networks</t>
+          <t>Introduction to Web Technologies, HTML5 Semantic Elements, Forms, Tables, CSS3 Selectors, Box Model, Responsive Design Basics</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -876,7 +921,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>The Network Core, Circuit switching and packet switching, Delay, Loss and throughput in packet switched networks</t>
+          <t>JavaScript ES6+, DOM Manipulation, Event Handling, Promises, Async/Await, Fetch API, JSON</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -899,7 +944,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Protocol Layers and their Service Models, IP stack, OSI Model</t>
+          <t>Server-side Programming with Node.js, Express.js, HTTP Request/Response Cycle, Middleware, REST API Design</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -922,7 +967,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Introduction to principles of Network Applications, The Web and HTTP types Persistent and Non-persistent</t>
+          <t>Database Connectivity, MongoDB CRUD Operations, Mongoose ODM, AJAX, Session and Cookie Management</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -945,7 +990,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Basic Networking Commands, Socket programming in Java</t>
+          <t>Build a Responsive Web Application using HTML5, CSS3, and JavaScript with Backend Integration</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -968,7 +1013,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Introduction to the Network, The Internet, The Network Edge, Network Topology, Types of Networks, The Network Core, Circuit switching and packet switching, Delay, Loss and throughput in packet switched networks, Protocol Layers and their Service Models, IP stack, OSI Model</t>
+          <t>HTML5, CSS3, JavaScript Fundamentals, Node.js, Express.js Basics, HTTP Protocol</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -991,7 +1036,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Introduction to the Network, The Internet, The Network Edge, Network Topology, Types of Networks, The Network Core, Circuit switching and packet switching, Delay, Loss and throughput in packet switched networks, Protocol Layers and their Service Models, IP stack, OSI Model, Introduction to principles of Network Applications, The Web and HTTP types Persistent and Non-persistent, FTP, Electronic Mail in the Internet with SMTP, POP3 and IMAP protocol, DNS - Routing, Caching</t>
+          <t>Full-Stack Web Development: Frontend (HTML/CSS/JS), Backend (Node.js/Express), Database (MongoDB), REST APIs, Web Security (XSS, CSRF), Deployment</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -1011,7 +1056,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C9"/>
+  <dimension ref="A1:D9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1027,6 +1072,11 @@
       </c>
       <c r="C1" t="inlineStr">
         <is>
+          <t>Curriculum</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
           <t>Strategies</t>
         </is>
       </c>
@@ -1041,6 +1091,11 @@
         <v>10</v>
       </c>
       <c r="C2" t="inlineStr">
+        <is>
+          <t>Introduction to DBMS, Database Architecture (1-Tier, 2-Tier, 3-Tier), Entity-Relationship Model, Entity Types, Attributes, Primary Keys</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
         <is>
           <t>Step 1: Re-read the topic from your lecture notes and highlight the 3 most important concepts.
 Step 2: Look up 2-3 solved examples from your textbook that are similar to the assignment problem.
@@ -1061,6 +1116,11 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
+          <t>Relational Model, Relational Algebra (Select, Project, Join), SQL: DDL (CREATE, ALTER, DROP), DML (INSERT, UPDATE, DELETE)</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
           <t>Step 1: Carefully re-read the problem statement and underline the key requirements.
 Step 2: Identify which algorithm, concept, or formula is being tested in this assignment.
 Step 3: Write pseudo-code or a rough outline before writing your actual solution.
@@ -1080,6 +1140,11 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
+          <t>Advanced SQL: Joins (Inner, Left, Right, Full Outer), Subqueries, Aggregation Functions, Views, Stored Procedures and Triggers</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
           <t>Step 1: List all topics covered in class since the course started and create a quick topic checklist.
 Step 2: Make flashcards for key definitions, formulas, and important terms for each topic.
 Step 3: Solve at least 4-5 practice questions per topic from your textbook or past quizzes.
@@ -1099,6 +1164,11 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
+          <t>Database Normalization, Functional Dependencies, Closure, 1NF, 2NF, 3NF, BCNF, Lossless Decomposition</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
           <t>Step 1: Review your Quiz 1 paper and fix every mistake to understand why you went wrong.
 Step 2: Focus on the current topic: write out the key algorithm or concept from memory twice.
 Step 3: Implement the required algorithm or technique in code and run it to verify correctness.
@@ -1118,6 +1188,11 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
+          <t>Transaction Management, ACID Properties, Serializability, Concurrency Control, Two-Phase Locking, Timestamp Ordering</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
           <t>Step 1: Draw diagrams or visual representations for each concept covered since Quiz 2.
 Step 2: Trace through at least 2 worked examples step-by-step for each key topic.
 Step 3: Code up at least 2 implementations from scratch without looking at your notes.
@@ -1136,6 +1211,11 @@
         <v>30</v>
       </c>
       <c r="C7" t="inlineStr">
+        <is>
+          <t>Database Design Project: ER Diagram to Relational Schema, SQL Query Optimization on real datasets</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
         <is>
           <t>Step 1: Go through all lab exercises from the semester and redo the ones you found difficult.
 Step 2: Practice writing code entirely from scratch for the most common lab tasks without copy-paste.
@@ -1157,6 +1237,11 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
+          <t>ER Modeling, Relational Model, SQL Commands, Normalization up to BCNF</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
           <t>Step 1: Create a one-page topic summary for every chapter or unit covered so far.
 Step 2: Attempt 2 complete past mid-exam papers under strict timed conditions.
 Step 3: Identify your 3 weakest topics from the mock attempts and spend extra time on them.
@@ -1176,6 +1261,11 @@
         <v>100</v>
       </c>
       <c r="C9" t="inlineStr">
+        <is>
+          <t>Complete DBMS: ER Design, SQL, Normalization, Transaction Management, Recovery Techniques, Indexing (B-Tree, Hash), Query Optimization</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
         <is>
           <t>Step 1: Build a 2-week revision schedule that covers every topic with more time for weak areas.
 Step 2: Prioritize topics by their exam weight and your current performance from your marks data.
@@ -1242,7 +1332,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Introduction to the Network, The Internet, The Network Edge, Network Topology, Types of Networks</t>
+          <t>Introduction to Python for Data Science, NumPy: Arrays, Matrix Operations, Broadcasting, Indexing and Slicing</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -1265,7 +1355,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>The Network Core, Circuit switching and packet switching, Delay, Loss and throughput in packet switched networks</t>
+          <t>Pandas: DataFrames, Series, Data Cleaning, Handling Missing Values, Data Merging and Reshaping</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -1288,7 +1378,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Protocol Layers and their Service Models, IP stack, OSI Model</t>
+          <t>Descriptive Statistics: Mean, Median, Mode, Variance, Standard Deviation, Percentiles, Correlation, Covariance</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -1311,7 +1401,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Introduction to principles of Network Applications, The Web and HTTP types Persistent and Non-persistent</t>
+          <t>Data Visualization: Matplotlib (Line, Bar, Histogram, Scatter), Seaborn (Heatmap, Pairplot, Box Plot), Plotly Basics</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -1334,7 +1424,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Basic Networking Commands, Socket programming in Java</t>
+          <t>Exploratory Data Analysis (EDA) on Real-World Dataset: cleaning, statistical summary, and visualization</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -1357,7 +1447,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Introduction to the Network, The Internet, The Network Edge, Network Topology, Types of Networks, The Network Core, Circuit switching and packet switching, Delay, Loss and throughput in packet switched networks, Protocol Layers and their Service Models, IP stack, OSI Model</t>
+          <t>Python Fundamentals, NumPy, Pandas DataFrames, Descriptive Statistics, Data Cleaning</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -1380,7 +1470,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Introduction to the Network, The Internet, The Network Edge, Network Topology, Types of Networks, The Network Core, Circuit switching and packet switching, Delay, Loss and throughput in packet switched networks, Protocol Layers and their Service Models, IP stack, OSI Model, Introduction to principles of Network Applications, The Web and HTTP types Persistent and Non-persistent, FTP, Electronic Mail in the Internet with SMTP, POP3 and IMAP protocol, DNS - Routing, Caching</t>
+          <t>End-to-End Data Analytics Pipeline: Data Collection, Preprocessing, EDA, Statistical Analysis, Visualization, Interpretation and Reporting</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -1400,7 +1490,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C9"/>
+  <dimension ref="A1:D9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1416,6 +1506,11 @@
       </c>
       <c r="C1" t="inlineStr">
         <is>
+          <t>Curriculum</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
           <t>Strategies</t>
         </is>
       </c>
@@ -1430,6 +1525,11 @@
         <v>10</v>
       </c>
       <c r="C2" t="inlineStr">
+        <is>
+          <t>Introduction to Statistical Learning, Bias-Variance Tradeoff, Overfitting vs Underfitting, Training/Validation/Test Split</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
         <is>
           <t>Step 1: Re-read the topic from your lecture notes and highlight the 3 most important concepts.
 Step 2: Look up 2-3 solved examples from your textbook that are similar to the assignment problem.
@@ -1450,6 +1550,11 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
+          <t>Linear Regression, Multiple Regression, Least Squares Method, Hypothesis Testing, R-Squared, Adjusted R-Squared</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
           <t>Step 1: Carefully re-read the problem statement and underline the key requirements.
 Step 2: Identify which algorithm, concept, or formula is being tested in this assignment.
 Step 3: Write pseudo-code or a rough outline before writing your actual solution.
@@ -1469,6 +1574,11 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
+          <t>Classification: k-Nearest Neighbors (kNN), Naive Bayes Classifier, Logistic Regression, Decision Boundary, ROC Curve, AUC</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
           <t>Step 1: List all topics covered in class since the course started and create a quick topic checklist.
 Step 2: Make flashcards for key definitions, formulas, and important terms for each topic.
 Step 3: Solve at least 4-5 practice questions per topic from your textbook or past quizzes.
@@ -1488,6 +1598,11 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
+          <t>Support Vector Machines (SVM), Kernel Functions (RBF, Polynomial), SVM for Classification and Regression (SVR)</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
           <t>Step 1: Review your Quiz 1 paper and fix every mistake to understand why you went wrong.
 Step 2: Focus on the current topic: write out the key algorithm or concept from memory twice.
 Step 3: Implement the required algorithm or technique in code and run it to verify correctness.
@@ -1507,6 +1622,11 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
+          <t>Unsupervised Learning: K-Means Clustering, Hierarchical Clustering (Dendrogram), DBSCAN, Principal Component Analysis (PCA)</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
           <t>Step 1: Draw diagrams or visual representations for each concept covered since Quiz 2.
 Step 2: Trace through at least 2 worked examples step-by-step for each key topic.
 Step 3: Code up at least 2 implementations from scratch without looking at your notes.
@@ -1525,6 +1645,11 @@
         <v>30</v>
       </c>
       <c r="C7" t="inlineStr">
+        <is>
+          <t>Implement and evaluate Regression and Classification models using scikit-learn on real datasets</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
         <is>
           <t>Step 1: Go through all lab exercises from the semester and redo the ones you found difficult.
 Step 2: Practice writing code entirely from scratch for the most common lab tasks without copy-paste.
@@ -1546,6 +1671,11 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
+          <t>Statistical Learning Theory, Linear Regression, Classification Algorithms, Model Evaluation Metrics</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
           <t>Step 1: Create a one-page topic summary for every chapter or unit covered so far.
 Step 2: Attempt 2 complete past mid-exam papers under strict timed conditions.
 Step 3: Identify your 3 weakest topics from the mock attempts and spend extra time on them.
@@ -1565,6 +1695,11 @@
         <v>100</v>
       </c>
       <c r="C9" t="inlineStr">
+        <is>
+          <t>Full ML Pipeline: Preprocessing, Feature Engineering, Supervised/Unsupervised Learning, Model Selection, Hyperparameter Tuning, Cross-Validation, Evaluation</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
         <is>
           <t>Step 1: Build a 2-week revision schedule that covers every topic with more time for weak areas.
 Step 2: Prioritize topics by their exam weight and your current performance from your marks data.
@@ -1631,7 +1766,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Introduction to the Network, The Internet, The Network Edge, Network Topology, Types of Networks</t>
+          <t>Introduction to Artificial Intelligence, Intelligent Agents, PEAS Framework, Types of Agents: Simple Reflex, Model-Based, Goal-Based, Utility-Based</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -1654,7 +1789,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>The Network Core, Circuit switching and packet switching, Delay, Loss and throughput in packet switched networks</t>
+          <t>Problem Solving by Search: State Space, BFS, DFS, Uniform Cost Search, Iterative Deepening DFS, Bidirectional Search</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -1677,7 +1812,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Protocol Layers and their Service Models, IP stack, OSI Model</t>
+          <t>Informed Search: Heuristic Functions, Greedy Best-First Search, A* Algorithm, Admissibility and Consistency, Hill Climbing</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -1700,7 +1835,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Introduction to principles of Network Applications, The Web and HTTP types Persistent and Non-persistent</t>
+          <t>Knowledge Representation: Propositional Logic, Wumpus World, First-Order Predicate Logic, Quantifiers, Inference Rules, Unification</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -1723,7 +1858,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Basic Networking Commands, Socket programming in Java</t>
+          <t>Implement BFS, DFS, A* Search Algorithms in Python; Solve 8-Puzzle and Maze problems</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -1746,7 +1881,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Introduction to the Network, The Internet, The Network Edge, Network Topology, Types of Networks, The Network Core, Circuit switching and packet switching, Delay, Loss and throughput in packet switched networks, Protocol Layers and their Service Models, IP stack, OSI Model</t>
+          <t>Intelligent Agents, Uninformed Search (BFS/DFS/UCS), Informed Search (A* /Greedy), Knowledge Representation</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -1769,7 +1904,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Introduction to the Network, The Internet, The Network Edge, Network Topology, Types of Networks, The Network Core, Circuit switching and packet switching, Delay, Loss and throughput in packet switched networks, Protocol Layers and their Service Models, IP stack, OSI Model, Introduction to principles of Network Applications, The Web and HTTP types Persistent and Non-persistent, FTP, Electronic Mail in the Internet with SMTP, POP3 and IMAP protocol, DNS - Routing, Caching</t>
+          <t>Complete AI: Search Strategies, Logic, Knowledge Representation and Reasoning, Planning (STRIPS), Uncertainty (Bayesian Networks), Learning Basics</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -1789,7 +1924,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C9"/>
+  <dimension ref="A1:D9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1805,6 +1940,11 @@
       </c>
       <c r="C1" t="inlineStr">
         <is>
+          <t>Curriculum</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
           <t>Strategies</t>
         </is>
       </c>
@@ -1819,6 +1959,11 @@
         <v>10</v>
       </c>
       <c r="C2" t="inlineStr">
+        <is>
+          <t>Introduction to Neural Networks, Biological Inspiration, Perceptron, Multi-Layer Perceptron (MLP), Activation Functions (ReLU, Sigmoid, Tanh, Softmax), Forward Propagation</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
         <is>
           <t>Step 1: Re-read the topic from your lecture notes and highlight the 3 most important concepts.
 Step 2: Look up 2-3 solved examples from your textbook that are similar to the assignment problem.
@@ -1839,6 +1984,11 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
+          <t>Backpropagation Algorithm, Computation Graph, Gradient Descent Variants (Batch, SGD, Mini-Batch), Optimizers: Adam, RMSprop, Momentum, Learning Rate Scheduling</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
           <t>Step 1: Carefully re-read the problem statement and underline the key requirements.
 Step 2: Identify which algorithm, concept, or formula is being tested in this assignment.
 Step 3: Write pseudo-code or a rough outline before writing your actual solution.
@@ -1858,6 +2008,11 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
+          <t>Convolutional Neural Networks (CNN): Convolution Layers, Pooling, Feature Maps, Padding, Stride, Architectures: LeNet, AlexNet, VGG, ResNet</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
           <t>Step 1: List all topics covered in class since the course started and create a quick topic checklist.
 Step 2: Make flashcards for key definitions, formulas, and important terms for each topic.
 Step 3: Solve at least 4-5 practice questions per topic from your textbook or past quizzes.
@@ -1877,6 +2032,11 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
+          <t>Recurrent Neural Networks (RNN): Vanishing Gradient Problem, Long Short-Term Memory (LSTM), Gated Recurrent Unit (GRU), Sequence-to-Sequence Models</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
           <t>Step 1: Review your Quiz 1 paper and fix every mistake to understand why you went wrong.
 Step 2: Focus on the current topic: write out the key algorithm or concept from memory twice.
 Step 3: Implement the required algorithm or technique in code and run it to verify correctness.
@@ -1896,6 +2056,11 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
+          <t>Transfer Learning, Fine-Tuning Pre-trained Models, Generative Adversarial Networks (GANs), Variational Autoencoders (VAE)</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
           <t>Step 1: Draw diagrams or visual representations for each concept covered since Quiz 2.
 Step 2: Trace through at least 2 worked examples step-by-step for each key topic.
 Step 3: Code up at least 2 implementations from scratch without looking at your notes.
@@ -1914,6 +2079,11 @@
         <v>30</v>
       </c>
       <c r="C7" t="inlineStr">
+        <is>
+          <t>Build and Train a CNN using TensorFlow/Keras for Image Classification (MNIST/CIFAR-10)</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
         <is>
           <t>Step 1: Go through all lab exercises from the semester and redo the ones you found difficult.
 Step 2: Practice writing code entirely from scratch for the most common lab tasks without copy-paste.
@@ -1935,6 +2105,11 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
+          <t>Neural Network Fundamentals, Backpropagation, CNN Architectures, RNN/LSTM Applications</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
           <t>Step 1: Create a one-page topic summary for every chapter or unit covered so far.
 Step 2: Attempt 2 complete past mid-exam papers under strict timed conditions.
 Step 3: Identify your 3 weakest topics from the mock attempts and spend extra time on them.
@@ -1954,6 +2129,11 @@
         <v>100</v>
       </c>
       <c r="C9" t="inlineStr">
+        <is>
+          <t>Advanced Deep Learning: Attention Mechanism, Transformer Architecture, BERT, GPT Basics, Autoencoders, GANs, Model Deployment with TensorFlow Serving</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
         <is>
           <t>Step 1: Build a 2-week revision schedule that covers every topic with more time for weak areas.
 Step 2: Prioritize topics by their exam weight and your current performance from your marks data.

</xml_diff>